<commit_message>
docs(ao-frdisi): bordereau — ligne câbles DC Bât. B déplacée des prestations communes vers la section BÂTIMENT B (item 16), renumérotation 1-30, totaux inchangés 4 166 600 HT / 4 999 920 TTC
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ao-frdisi/releve-2026-07-27/ENVOI_ACCORDIA_MAJ/04 - Bordereau des prix - REVISE 27-07.xlsx
+++ b/docs/ao-frdisi/releve-2026-07-27/ENVOI_ACCORDIA_MAJ/04 - Bordereau des prix - REVISE 27-07.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://atlenciax-my.sharepoint.com/personal/redakasri_atlenciax_onmicrosoft_com/Documents/TAQINOR/AO FRDISI - Solaire Mohammedia 2026/ENVOI ACCORDIA - FINAL 27-07/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_85E66461937B9CDFEF56F476522D1E7DD9FF6B6F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_E0F23B8E5052B8DEEF56F476522D1E7DD9FFB826" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5760" yWindow="3312" windowWidth="17280" windowHeight="8928" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bordereau" sheetId="1" r:id="rId1"/>
@@ -71,7 +71,7 @@
     <t>Onduleurs hybrides triphasés 50 kW Deye SUN-50K-SG01HP3-EU-BM4, y compris compteur zéro injection Eastron SDM630-MCT + TC, pose et mise en service</t>
   </si>
   <si>
-    <t>Batteries LFP haute tension Deye BOS-G (modules 5,12 kWh + coffret HV HVB750V/100A), y compris pose, protections et mise en service</t>
+    <t>Batteries LFP haute tension Deye BOS-B Pro (packs 16,08 kWh BOS-B-Pack16-A3 + coffret HV BOS-B-PDU-2-A + racks), y compris pose, protections et mise en service</t>
   </si>
   <si>
     <t>kWh</t>
@@ -104,6 +104,9 @@
     <t>TGPV B et couplage au TGBT existant du bâtiment, y compris adaptation</t>
   </si>
   <si>
+    <t>Câbles solaires 6 mm² EN 50618, chemins de câbles UV avec couvercle, mise à la terre et liaisons équipotentielles (aile en arc) — quote-part de l'enveloppe câbles DC projet (10 km × 15 000 DH HT/km)</t>
+  </si>
+  <si>
     <t>BÂTIMENT C — ÉCOLE SUPTECH — 180,0 kWc</t>
   </si>
   <si>
@@ -117,9 +120,6 @@
   </si>
   <si>
     <t>Études d'exécution complètes (note de calcul, calepinage, schémas), note de calcul vent/structure par BET, visa bureau de contrôle agréé, dossier d'exécution</t>
-  </si>
-  <si>
-    <t>Câbles solaires, chemins de câbles, mise à la terre — Bâtiment B (aile en arc) — quote-part de l'enveloppe câbles DC projet (10 km × 15 000 DH HT/km)</t>
   </si>
   <si>
     <t>Liaison électrique et communication inter-sites (U1000 AR2V 3x240+120 mm² alu enterré sous fourreau TPC Ø160, fibre optique 8 brins, protections et compteurs bidirectionnels aux deux extrémités, génie civil de tranchée)</t>
@@ -849,7 +849,7 @@
         <v>2950</v>
       </c>
       <c r="F15" s="5">
-        <f t="shared" ref="F15:F20" si="1">D15*E15</f>
+        <f t="shared" ref="F15:F21" si="1">D15*E15</f>
         <v>354000</v>
       </c>
     </row>
@@ -958,56 +958,56 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="12" t="s">
+    <row r="21" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="2">
+        <v>16</v>
+      </c>
+      <c r="B21" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B21" s="9"/>
-      <c r="C21" s="9"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="9"/>
-      <c r="F21" s="9"/>
+      <c r="C21" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D21" s="2">
+        <v>1</v>
+      </c>
+      <c r="E21" s="4">
+        <v>45000</v>
+      </c>
+      <c r="F21" s="5">
+        <f t="shared" si="1"/>
+        <v>45000</v>
+      </c>
     </row>
     <row r="22" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="2">
-        <v>16</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D22" s="2">
-        <v>288</v>
-      </c>
-      <c r="E22" s="4">
-        <v>2950</v>
-      </c>
-      <c r="F22" s="5">
-        <f t="shared" ref="F22:F30" si="2">D22*E22</f>
-        <v>849600</v>
-      </c>
+      <c r="A22" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="B22" s="9"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
     </row>
     <row r="23" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
         <v>17</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D23" s="2">
-        <v>3</v>
+        <v>288</v>
       </c>
       <c r="E23" s="4">
-        <v>78000</v>
+        <v>2950</v>
       </c>
       <c r="F23" s="5">
-        <f t="shared" si="2"/>
-        <v>234000</v>
+        <f t="shared" ref="F23:F31" si="2">D23*E23</f>
+        <v>849600</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.3">
@@ -1015,20 +1015,20 @@
         <v>18</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D24" s="2">
-        <v>92</v>
+        <v>3</v>
       </c>
       <c r="E24" s="4">
-        <v>2600</v>
+        <v>78000</v>
       </c>
       <c r="F24" s="5">
         <f t="shared" si="2"/>
-        <v>239200</v>
+        <v>234000</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.3">
@@ -1036,20 +1036,20 @@
         <v>19</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D25" s="2">
-        <v>3</v>
+        <v>92</v>
       </c>
       <c r="E25" s="4">
-        <v>4500</v>
+        <v>2600</v>
       </c>
       <c r="F25" s="5">
         <f t="shared" si="2"/>
-        <v>13500</v>
+        <v>239200</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.3">
@@ -1057,7 +1057,7 @@
         <v>20</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>10</v>
@@ -1066,11 +1066,11 @@
         <v>3</v>
       </c>
       <c r="E26" s="4">
-        <v>8500</v>
+        <v>4500</v>
       </c>
       <c r="F26" s="5">
         <f t="shared" si="2"/>
-        <v>25500</v>
+        <v>13500</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.3">
@@ -1078,20 +1078,20 @@
         <v>21</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="D27" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E27" s="4">
-        <v>15000</v>
+        <v>8500</v>
       </c>
       <c r="F27" s="5">
         <f t="shared" si="2"/>
-        <v>15000</v>
+        <v>25500</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.3">
@@ -1108,11 +1108,11 @@
         <v>1</v>
       </c>
       <c r="E28" s="4">
-        <v>45000</v>
+        <v>15000</v>
       </c>
       <c r="F28" s="5">
         <f t="shared" si="2"/>
-        <v>45000</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.3">
@@ -1120,20 +1120,20 @@
         <v>23</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D29" s="2">
         <v>1</v>
       </c>
       <c r="E29" s="4">
-        <v>50000</v>
+        <v>45000</v>
       </c>
       <c r="F29" s="5">
         <f t="shared" si="2"/>
-        <v>50000</v>
+        <v>45000</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.3">
@@ -1141,7 +1141,7 @@
         <v>24</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>10</v>
@@ -1150,43 +1150,43 @@
         <v>1</v>
       </c>
       <c r="E30" s="4">
-        <v>39500</v>
+        <v>50000</v>
       </c>
       <c r="F30" s="5">
         <f t="shared" si="2"/>
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="2">
+        <v>25</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D31" s="2">
+        <v>1</v>
+      </c>
+      <c r="E31" s="4">
         <v>39500</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="B31" s="9"/>
-      <c r="C31" s="9"/>
-      <c r="D31" s="9"/>
-      <c r="E31" s="9"/>
-      <c r="F31" s="9"/>
+      <c r="F31" s="5">
+        <f t="shared" si="2"/>
+        <v>39500</v>
+      </c>
     </row>
     <row r="32" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="2">
-        <v>25</v>
-      </c>
-      <c r="B32" s="3" t="s">
+      <c r="A32" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="C32" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D32" s="2">
-        <v>1</v>
-      </c>
-      <c r="E32" s="4">
-        <v>262000</v>
-      </c>
-      <c r="F32" s="5">
-        <f t="shared" ref="F32:F37" si="3">D32*E32</f>
-        <v>262000</v>
-      </c>
+      <c r="B32" s="9"/>
+      <c r="C32" s="9"/>
+      <c r="D32" s="9"/>
+      <c r="E32" s="9"/>
+      <c r="F32" s="9"/>
     </row>
     <row r="33" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2">
@@ -1202,11 +1202,11 @@
         <v>1</v>
       </c>
       <c r="E33" s="4">
-        <v>45000</v>
+        <v>262000</v>
       </c>
       <c r="F33" s="5">
-        <f t="shared" si="3"/>
-        <v>45000</v>
+        <f>D33*E33</f>
+        <v>262000</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.3">
@@ -1226,7 +1226,7 @@
         <v>1500</v>
       </c>
       <c r="F34" s="5">
-        <f t="shared" si="3"/>
+        <f>D34*E34</f>
         <v>225000</v>
       </c>
     </row>
@@ -1247,7 +1247,7 @@
         <v>200000</v>
       </c>
       <c r="F35" s="5">
-        <f t="shared" si="3"/>
+        <f>D35*E35</f>
         <v>200000</v>
       </c>
     </row>
@@ -1268,7 +1268,7 @@
         <v>120000</v>
       </c>
       <c r="F36" s="5">
-        <f t="shared" si="3"/>
+        <f>D36*E36</f>
         <v>120000</v>
       </c>
     </row>
@@ -1289,7 +1289,7 @@
         <v>70000</v>
       </c>
       <c r="F37" s="5">
-        <f t="shared" si="3"/>
+        <f>D37*E37</f>
         <v>70000</v>
       </c>
     </row>
@@ -1368,9 +1368,9 @@
     <mergeCell ref="A14:F14"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A45:F45"/>
-    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A32:F32"/>
+    <mergeCell ref="A22:F22"/>
     <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A21:F21"/>
     <mergeCell ref="A43:F43"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>